<commit_message>
feat: add excel manipulation service
</commit_message>
<xml_diff>
--- a/templates/employees.xlsx
+++ b/templates/employees.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minamalak/Repos/billing-automation/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1217690-7D57-6B4E-926C-9A5B3F98F488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B548C5-F8D5-1A48-BC65-72631D70BD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,22 +53,22 @@
     <t>joiningDate</t>
   </si>
   <si>
-    <t>Mina Malak1</t>
-  </si>
-  <si>
     <t>Youstina Ayman2</t>
   </si>
   <si>
     <t>2 Shoubra street</t>
   </si>
   <si>
-    <t>2 EL Harm Street</t>
-  </si>
-  <si>
     <t>mkl@gh.cm23</t>
   </si>
   <si>
-    <t>m@x.ckl45</t>
+    <t>Mina Malak</t>
+  </si>
+  <si>
+    <t>1 Amin Hamada</t>
+  </si>
+  <si>
+    <t>minamalak6300@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -496,19 +496,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2">
-        <v>3010</v>
+        <v>1500</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2">
-        <v>12938494599</v>
+        <v>1226530946</v>
       </c>
       <c r="E2" s="2">
-        <v>45507</v>
+        <v>45505</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -516,13 +516,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3">
         <v>2010</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3">
         <v>12939448488</v>
@@ -531,7 +531,7 @@
         <v>44994</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>